<commit_message>
Póstlisti: sér dálkur fyrir íbúðarnúmer í fjölbýli
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fts7wXaAbvyJ2CRF93qGGq
</commit_message>
<xml_diff>
--- a/svif_postlisti_vika1.xlsx
+++ b/svif_postlisti_vika1.xlsx
@@ -417,14 +417,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E160"/>
+  <dimension ref="A1:F160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -440,15 +441,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Íbúð</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Póstnúmer</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Staður</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Hverfanúmer</t>
         </is>
@@ -465,15 +471,16 @@
           <t>Bergþórugata 7</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="n">
         <v>101</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -486,15 +493,16 @@
           <t>Bragagata 33</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="n">
         <v>101</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -507,15 +515,20 @@
           <t>Grettisgata 46, íbúð 0302</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0302</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
         <v>101</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -528,15 +541,20 @@
           <t>Leifsgata 18, íbúð 0101</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
         <v>101</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -549,15 +567,16 @@
           <t>Bauganes 3</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="n">
         <v>102</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -570,15 +589,16 @@
           <t>Reykjavíkurvegur 23</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="n">
         <v>102</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -591,15 +611,16 @@
           <t>Hvassaleiti 103</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="n">
         <v>103</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -612,15 +633,16 @@
           <t>Drekavogur 14</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="n">
         <v>104</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -633,15 +655,16 @@
           <t>Efstasund 64</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
         <v>104</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -654,15 +677,16 @@
           <t>Kambsvegur 11</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="n">
         <v>104</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -675,15 +699,16 @@
           <t>Kleppsvegur 94</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="n">
         <v>104</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -696,15 +721,16 @@
           <t>Skipasund 77</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="n">
         <v>104</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -717,15 +743,20 @@
           <t>Barmahlíð 23, íbúð 0201</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>0201</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
         <v>105</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -738,15 +769,20 @@
           <t>Birkihlíð 42, íbúð 0101</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
         <v>105</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -759,15 +795,20 @@
           <t>Bólstaðarhlíð 48, íbúð 0201</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0201</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
         <v>105</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -780,15 +821,20 @@
           <t>Bólstaðarhlíð 5, íbúð 0101</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
         <v>105</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -801,15 +847,20 @@
           <t>Laugarnesvegur 112, íbúð 0105</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0105</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
         <v>105</v>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -822,15 +873,20 @@
           <t>Mávahlíð 11, íbúð 0101</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
         <v>105</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -843,15 +899,16 @@
           <t>Otrateigur 18</t>
         </is>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="n">
         <v>105</v>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -864,15 +921,20 @@
           <t>Rauðalækur 51, íbúð 0101</t>
         </is>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
         <v>105</v>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -885,15 +947,20 @@
           <t>Skipholt 24, íbúð 0201</t>
         </is>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>0201</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
         <v>105</v>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -906,15 +973,20 @@
           <t>Stigahlíð 4, íbúð 0402</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>0402</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
         <v>105</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -927,15 +999,16 @@
           <t>Ásholt 28</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
         <v>105</v>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -948,15 +1021,20 @@
           <t>Hagamelur 48, íbúð 0101</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
         <v>107</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -969,15 +1047,20 @@
           <t>Tómasarhagi 36, íbúð 0101</t>
         </is>
       </c>
-      <c r="C26" t="n">
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
         <v>107</v>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -990,15 +1073,20 @@
           <t>Víðimelur 30, íbúð 0201</t>
         </is>
       </c>
-      <c r="C27" t="n">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>0201</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
         <v>107</v>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1011,15 +1099,16 @@
           <t>Heiðargerði 3</t>
         </is>
       </c>
-      <c r="C28" t="n">
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="n">
         <v>108</v>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1032,15 +1121,16 @@
           <t>Heiðargerði 33</t>
         </is>
       </c>
-      <c r="C29" t="n">
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="n">
         <v>108</v>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1053,15 +1143,16 @@
           <t>Heiðargerði 43</t>
         </is>
       </c>
-      <c r="C30" t="n">
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="n">
         <v>108</v>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1074,15 +1165,16 @@
           <t>Háaleitisbraut 93</t>
         </is>
       </c>
-      <c r="C31" t="n">
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="n">
         <v>108</v>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1095,15 +1187,16 @@
           <t>Kúrland 26</t>
         </is>
       </c>
-      <c r="C32" t="n">
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="n">
         <v>108</v>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1116,15 +1209,16 @@
           <t>Ljósaland 3</t>
         </is>
       </c>
-      <c r="C33" t="n">
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
         <v>108</v>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1137,15 +1231,20 @@
           <t>Álftamýri 36, íbúð 0203</t>
         </is>
       </c>
-      <c r="C34" t="n">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>0203</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
         <v>108</v>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1158,15 +1257,16 @@
           <t>Ásgarður 123</t>
         </is>
       </c>
-      <c r="C35" t="n">
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="n">
         <v>108</v>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1179,15 +1279,16 @@
           <t>Bakkasel 25</t>
         </is>
       </c>
-      <c r="C36" t="n">
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="n">
         <v>109</v>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1200,15 +1301,16 @@
           <t>Engjasel 66</t>
         </is>
       </c>
-      <c r="C37" t="n">
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="n">
         <v>109</v>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1221,15 +1323,16 @@
           <t>Engjasel 82</t>
         </is>
       </c>
-      <c r="C38" t="n">
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="n">
         <v>109</v>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1242,15 +1345,20 @@
           <t>Eyjabakki 7, íbúð 0202</t>
         </is>
       </c>
-      <c r="C39" t="n">
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>0202</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
         <v>109</v>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1263,15 +1371,20 @@
           <t>Ferjubakki 2, íbúð 0202</t>
         </is>
       </c>
-      <c r="C40" t="n">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>0202</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
         <v>109</v>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1284,15 +1397,16 @@
           <t>Látrasel 12</t>
         </is>
       </c>
-      <c r="C41" t="n">
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="n">
         <v>109</v>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1305,15 +1419,16 @@
           <t>Seljabraut 46</t>
         </is>
       </c>
-      <c r="C42" t="n">
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="n">
         <v>109</v>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1326,15 +1441,16 @@
           <t>Strýtusel 10</t>
         </is>
       </c>
-      <c r="C43" t="n">
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="n">
         <v>109</v>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1347,15 +1463,16 @@
           <t>Strýtusel 13</t>
         </is>
       </c>
-      <c r="C44" t="n">
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="n">
         <v>109</v>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1368,15 +1485,16 @@
           <t>Stuðlasel 6</t>
         </is>
       </c>
-      <c r="C45" t="n">
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="n">
         <v>109</v>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1389,15 +1507,16 @@
           <t>Víkurbakki 8</t>
         </is>
       </c>
-      <c r="C46" t="n">
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="n">
         <v>109</v>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1410,15 +1529,16 @@
           <t>Eyktarás 15</t>
         </is>
       </c>
-      <c r="C47" t="n">
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="n">
         <v>110</v>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1431,15 +1551,20 @@
           <t>Hraunbær 158, íbúð 0301</t>
         </is>
       </c>
-      <c r="C48" t="n">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>0301</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
         <v>110</v>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1452,15 +1577,16 @@
           <t>Seiðakvísl 5</t>
         </is>
       </c>
-      <c r="C49" t="n">
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
         <v>110</v>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1473,15 +1599,16 @@
           <t>Þykkvibær 4</t>
         </is>
       </c>
-      <c r="C50" t="n">
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="n">
         <v>110</v>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1494,15 +1621,16 @@
           <t>Hamraberg 30</t>
         </is>
       </c>
-      <c r="C51" t="n">
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="n">
         <v>111</v>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1515,15 +1643,16 @@
           <t>Keilufell 4</t>
         </is>
       </c>
-      <c r="C52" t="n">
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="n">
         <v>111</v>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1536,15 +1665,16 @@
           <t>Torfufell 16</t>
         </is>
       </c>
-      <c r="C53" t="n">
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="n">
         <v>111</v>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1557,15 +1687,20 @@
           <t>Vesturberg 120, íbúð 0203</t>
         </is>
       </c>
-      <c r="C54" t="n">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>0203</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
         <v>111</v>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1578,15 +1713,16 @@
           <t>Vesturberg 97</t>
         </is>
       </c>
-      <c r="C55" t="n">
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="n">
         <v>111</v>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1599,15 +1735,20 @@
           <t>Æsufell 6, íbúð 0706</t>
         </is>
       </c>
-      <c r="C56" t="n">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>0706</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
         <v>111</v>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1620,15 +1761,16 @@
           <t>Fannafold 4</t>
         </is>
       </c>
-      <c r="C57" t="n">
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="n">
         <v>112</v>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1641,15 +1783,16 @@
           <t>Funafold 12</t>
         </is>
       </c>
-      <c r="C58" t="n">
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="n">
         <v>112</v>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1662,15 +1805,16 @@
           <t>Þorláksgeisli 46</t>
         </is>
       </c>
-      <c r="C59" t="n">
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="n">
         <v>113</v>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1683,15 +1827,16 @@
           <t>Vindheimar</t>
         </is>
       </c>
-      <c r="C60" t="n">
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="n">
         <v>162</v>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1704,15 +1849,16 @@
           <t>Lindarbraut 17</t>
         </is>
       </c>
-      <c r="C61" t="n">
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="n">
         <v>170</v>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>Seltjarnarnes</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1725,15 +1871,16 @@
           <t>Lindarbraut 24</t>
         </is>
       </c>
-      <c r="C62" t="n">
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="n">
         <v>170</v>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>Seltjarnarnes</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1746,15 +1893,16 @@
           <t>Melabraut 48</t>
         </is>
       </c>
-      <c r="C63" t="n">
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="n">
         <v>170</v>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Seltjarnarnes</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1767,15 +1915,16 @@
           <t>Nesbali 20</t>
         </is>
       </c>
-      <c r="C64" t="n">
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="n">
         <v>170</v>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>Seltjarnarnes</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1788,15 +1937,16 @@
           <t>Nesbali 25</t>
         </is>
       </c>
-      <c r="C65" t="n">
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="n">
         <v>170</v>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>Seltjarnarnes</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1809,15 +1959,16 @@
           <t>Sefgarðar 20</t>
         </is>
       </c>
-      <c r="C66" t="n">
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="n">
         <v>170</v>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>Seltjarnarnes</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1830,15 +1981,16 @@
           <t>Sefgarðar 28</t>
         </is>
       </c>
-      <c r="C67" t="n">
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="n">
         <v>170</v>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="E67" t="inlineStr">
         <is>
           <t>Seltjarnarnes</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1851,15 +2003,16 @@
           <t>Sævargarðar 7</t>
         </is>
       </c>
-      <c r="C68" t="n">
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="n">
         <v>170</v>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="E68" t="inlineStr">
         <is>
           <t>Seltjarnarnes</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1872,15 +2025,16 @@
           <t>Brekkugata 19</t>
         </is>
       </c>
-      <c r="C69" t="n">
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="n">
         <v>190</v>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>Vogar</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1893,15 +2047,16 @@
           <t>Heiðargerði 16</t>
         </is>
       </c>
-      <c r="C70" t="n">
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="n">
         <v>190</v>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>Vogar</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1914,15 +2069,16 @@
           <t>Vogagerði 17</t>
         </is>
       </c>
-      <c r="C71" t="n">
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="n">
         <v>190</v>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="E71" t="inlineStr">
         <is>
           <t>Vogar</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1935,15 +2091,16 @@
           <t>Bræðratunga 24</t>
         </is>
       </c>
-      <c r="C72" t="n">
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="n">
         <v>200</v>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="E72" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1956,15 +2113,16 @@
           <t>Daltún 17</t>
         </is>
       </c>
-      <c r="C73" t="n">
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="n">
         <v>200</v>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1977,15 +2135,20 @@
           <t>Fagrabrekka 25, íbúð 0101</t>
         </is>
       </c>
-      <c r="C74" t="n">
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
         <v>200</v>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1998,15 +2161,16 @@
           <t>Fagrihjalli 10</t>
         </is>
       </c>
-      <c r="C75" t="n">
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="n">
         <v>200</v>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2019,15 +2183,16 @@
           <t>Hlíðarvegur 6</t>
         </is>
       </c>
-      <c r="C76" t="n">
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="n">
         <v>200</v>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2040,15 +2205,16 @@
           <t>Hlíðarvegur 61</t>
         </is>
       </c>
-      <c r="C77" t="n">
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="n">
         <v>200</v>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2061,15 +2227,20 @@
           <t>Kjarrhólmi 6, íbúð 0302</t>
         </is>
       </c>
-      <c r="C78" t="n">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>0302</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
         <v>200</v>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2082,15 +2253,16 @@
           <t>Kópavogsbraut 63</t>
         </is>
       </c>
-      <c r="C79" t="n">
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="n">
         <v>200</v>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="E79" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2103,15 +2275,16 @@
           <t>Lyngbrekka 23</t>
         </is>
       </c>
-      <c r="C80" t="n">
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="n">
         <v>200</v>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="E80" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2124,15 +2297,16 @@
           <t>Þinghólsbraut 8</t>
         </is>
       </c>
-      <c r="C81" t="n">
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="n">
         <v>200</v>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="E81" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2145,15 +2319,16 @@
           <t>Aratún 28</t>
         </is>
       </c>
-      <c r="C82" t="n">
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="n">
         <v>210</v>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="E82" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2166,15 +2341,16 @@
           <t>Bæjargil 110</t>
         </is>
       </c>
-      <c r="C83" t="n">
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="n">
         <v>210</v>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="E83" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2187,15 +2363,16 @@
           <t>Efstilundur 8</t>
         </is>
       </c>
-      <c r="C84" t="n">
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="n">
         <v>210</v>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="E84" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2208,15 +2385,16 @@
           <t>Faxatún 5</t>
         </is>
       </c>
-      <c r="C85" t="n">
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="n">
         <v>210</v>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="E85" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2229,15 +2407,16 @@
           <t>Furulundur 2</t>
         </is>
       </c>
-      <c r="C86" t="n">
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="n">
         <v>210</v>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2250,15 +2429,16 @@
           <t>Hlíðarbyggð 3</t>
         </is>
       </c>
-      <c r="C87" t="n">
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="n">
         <v>210</v>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="E87" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2271,15 +2451,16 @@
           <t>Hlíðarbyggð 33</t>
         </is>
       </c>
-      <c r="C88" t="n">
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="n">
         <v>210</v>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="E88" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2292,15 +2473,20 @@
           <t>Hrísmóar 1, íbúð 0401</t>
         </is>
       </c>
-      <c r="C89" t="n">
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>0401</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
         <v>210</v>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="E89" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2313,15 +2499,16 @@
           <t>Kjarrmóar 11</t>
         </is>
       </c>
-      <c r="C90" t="n">
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="n">
         <v>210</v>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="E90" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2334,15 +2521,16 @@
           <t>Kjarrmóar 23</t>
         </is>
       </c>
-      <c r="C91" t="n">
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="n">
         <v>210</v>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2355,15 +2543,16 @@
           <t>Langafit 26</t>
         </is>
       </c>
-      <c r="C92" t="n">
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="n">
         <v>210</v>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="E92" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2376,15 +2565,16 @@
           <t>Lindarflöt 40</t>
         </is>
       </c>
-      <c r="C93" t="n">
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="n">
         <v>210</v>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2397,15 +2587,16 @@
           <t>Markarflöt 9</t>
         </is>
       </c>
-      <c r="C94" t="n">
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="n">
         <v>210</v>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="E94" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2418,15 +2609,16 @@
           <t>Móaflöt 12</t>
         </is>
       </c>
-      <c r="C95" t="n">
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="n">
         <v>210</v>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="E95" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2439,15 +2631,16 @@
           <t>Naustahlein 26</t>
         </is>
       </c>
-      <c r="C96" t="n">
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="n">
         <v>210</v>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="E96" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2460,15 +2653,16 @@
           <t>Smáraflöt 45</t>
         </is>
       </c>
-      <c r="C97" t="n">
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="n">
         <v>210</v>
       </c>
-      <c r="D97" t="inlineStr">
+      <c r="E97" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2481,15 +2675,20 @@
           <t>Arnarhraun 9, íbúð 0201</t>
         </is>
       </c>
-      <c r="C98" t="n">
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>0201</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
         <v>220</v>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="E98" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2502,15 +2701,16 @@
           <t>Brekkuhvammur 16</t>
         </is>
       </c>
-      <c r="C99" t="n">
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="n">
         <v>220</v>
       </c>
-      <c r="D99" t="inlineStr">
+      <c r="E99" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2523,15 +2723,16 @@
           <t>Erluhraun 3</t>
         </is>
       </c>
-      <c r="C100" t="n">
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="n">
         <v>220</v>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="E100" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2544,15 +2745,16 @@
           <t>Hellubraut 9</t>
         </is>
       </c>
-      <c r="C101" t="n">
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="n">
         <v>220</v>
       </c>
-      <c r="D101" t="inlineStr">
+      <c r="E101" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2565,15 +2767,16 @@
           <t>Hjallabraut 70</t>
         </is>
       </c>
-      <c r="C102" t="n">
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="n">
         <v>220</v>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="E102" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2586,15 +2789,16 @@
           <t>Kirkjuvegur 13</t>
         </is>
       </c>
-      <c r="C103" t="n">
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="n">
         <v>220</v>
       </c>
-      <c r="D103" t="inlineStr">
+      <c r="E103" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2607,15 +2811,16 @@
           <t>Kirkjuvegur 3</t>
         </is>
       </c>
-      <c r="C104" t="n">
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="n">
         <v>220</v>
       </c>
-      <c r="D104" t="inlineStr">
+      <c r="E104" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2628,15 +2833,16 @@
           <t>Klausturhvammur 30</t>
         </is>
       </c>
-      <c r="C105" t="n">
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="n">
         <v>220</v>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="E105" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2649,15 +2855,16 @@
           <t>Langeyrarvegur 16</t>
         </is>
       </c>
-      <c r="C106" t="n">
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="n">
         <v>220</v>
       </c>
-      <c r="D106" t="inlineStr">
+      <c r="E106" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2670,15 +2877,16 @@
           <t>Mávahraun 1</t>
         </is>
       </c>
-      <c r="C107" t="n">
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="n">
         <v>220</v>
       </c>
-      <c r="D107" t="inlineStr">
+      <c r="E107" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2691,15 +2899,16 @@
           <t>Selvogsgata 20</t>
         </is>
       </c>
-      <c r="C108" t="n">
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="n">
         <v>220</v>
       </c>
-      <c r="D108" t="inlineStr">
+      <c r="E108" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2712,15 +2921,16 @@
           <t>Smyrlahraun 19</t>
         </is>
       </c>
-      <c r="C109" t="n">
+      <c r="C109" t="inlineStr"/>
+      <c r="D109" t="n">
         <v>220</v>
       </c>
-      <c r="D109" t="inlineStr">
+      <c r="E109" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2733,15 +2943,16 @@
           <t>Smárahvammur 4</t>
         </is>
       </c>
-      <c r="C110" t="n">
+      <c r="C110" t="inlineStr"/>
+      <c r="D110" t="n">
         <v>220</v>
       </c>
-      <c r="D110" t="inlineStr">
+      <c r="E110" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2754,15 +2965,16 @@
           <t>Suðurgata 56</t>
         </is>
       </c>
-      <c r="C111" t="n">
+      <c r="C111" t="inlineStr"/>
+      <c r="D111" t="n">
         <v>220</v>
       </c>
-      <c r="D111" t="inlineStr">
+      <c r="E111" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2775,15 +2987,16 @@
           <t>Öldugata 26</t>
         </is>
       </c>
-      <c r="C112" t="n">
+      <c r="C112" t="inlineStr"/>
+      <c r="D112" t="n">
         <v>220</v>
       </c>
-      <c r="D112" t="inlineStr">
+      <c r="E112" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2796,15 +3009,16 @@
           <t>Ölduslóð 43</t>
         </is>
       </c>
-      <c r="C113" t="n">
+      <c r="C113" t="inlineStr"/>
+      <c r="D113" t="n">
         <v>220</v>
       </c>
-      <c r="D113" t="inlineStr">
+      <c r="E113" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2817,15 +3031,16 @@
           <t>Axlarás 39</t>
         </is>
       </c>
-      <c r="C114" t="n">
+      <c r="C114" t="inlineStr"/>
+      <c r="D114" t="n">
         <v>221</v>
       </c>
-      <c r="D114" t="inlineStr">
+      <c r="E114" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2838,15 +3053,16 @@
           <t>Glitvellir 14</t>
         </is>
       </c>
-      <c r="C115" t="n">
+      <c r="C115" t="inlineStr"/>
+      <c r="D115" t="n">
         <v>221</v>
       </c>
-      <c r="D115" t="inlineStr">
+      <c r="E115" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2859,15 +3075,20 @@
           <t>Hringhamar 8, íbúð 0202</t>
         </is>
       </c>
-      <c r="C116" t="n">
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>0202</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
         <v>221</v>
       </c>
-      <c r="D116" t="inlineStr">
+      <c r="E116" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2880,15 +3101,16 @@
           <t>Stuðlaberg 48</t>
         </is>
       </c>
-      <c r="C117" t="n">
+      <c r="C117" t="inlineStr"/>
+      <c r="D117" t="n">
         <v>221</v>
       </c>
-      <c r="D117" t="inlineStr">
+      <c r="E117" t="inlineStr">
         <is>
           <t>Hafnarfjörður</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2901,15 +3123,16 @@
           <t>Helguvík</t>
         </is>
       </c>
-      <c r="C118" t="n">
+      <c r="C118" t="inlineStr"/>
+      <c r="D118" t="n">
         <v>225</v>
       </c>
-      <c r="D118" t="inlineStr">
+      <c r="E118" t="inlineStr">
         <is>
           <t>Garðabær (Álftanes)</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2922,15 +3145,16 @@
           <t>Víðiholt 10</t>
         </is>
       </c>
-      <c r="C119" t="n">
+      <c r="C119" t="inlineStr"/>
+      <c r="D119" t="n">
         <v>225</v>
       </c>
-      <c r="D119" t="inlineStr">
+      <c r="E119" t="inlineStr">
         <is>
           <t>Garðabær (Álftanes)</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2943,15 +3167,16 @@
           <t>Faxabraut 31A</t>
         </is>
       </c>
-      <c r="C120" t="n">
+      <c r="C120" t="inlineStr"/>
+      <c r="D120" t="n">
         <v>230</v>
       </c>
-      <c r="D120" t="inlineStr">
+      <c r="E120" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2964,15 +3189,16 @@
           <t>Freyjuvellir 5</t>
         </is>
       </c>
-      <c r="C121" t="n">
+      <c r="C121" t="inlineStr"/>
+      <c r="D121" t="n">
         <v>230</v>
       </c>
-      <c r="D121" t="inlineStr">
+      <c r="E121" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2985,15 +3211,16 @@
           <t>Freyjuvellir 9</t>
         </is>
       </c>
-      <c r="C122" t="n">
+      <c r="C122" t="inlineStr"/>
+      <c r="D122" t="n">
         <v>230</v>
       </c>
-      <c r="D122" t="inlineStr">
+      <c r="E122" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3006,15 +3233,16 @@
           <t>Hafnargata 70</t>
         </is>
       </c>
-      <c r="C123" t="n">
+      <c r="C123" t="inlineStr"/>
+      <c r="D123" t="n">
         <v>230</v>
       </c>
-      <c r="D123" t="inlineStr">
+      <c r="E123" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3027,15 +3255,16 @@
           <t>Heiðarbraut 1E</t>
         </is>
       </c>
-      <c r="C124" t="n">
+      <c r="C124" t="inlineStr"/>
+      <c r="D124" t="n">
         <v>230</v>
       </c>
-      <c r="D124" t="inlineStr">
+      <c r="E124" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3048,15 +3277,16 @@
           <t>Heiðarvegur 21A</t>
         </is>
       </c>
-      <c r="C125" t="n">
+      <c r="C125" t="inlineStr"/>
+      <c r="D125" t="n">
         <v>230</v>
       </c>
-      <c r="D125" t="inlineStr">
+      <c r="E125" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3069,15 +3299,16 @@
           <t>Háaleiti 31</t>
         </is>
       </c>
-      <c r="C126" t="n">
+      <c r="C126" t="inlineStr"/>
+      <c r="D126" t="n">
         <v>230</v>
       </c>
-      <c r="D126" t="inlineStr">
+      <c r="E126" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3090,15 +3321,16 @@
           <t>Háteigur 20</t>
         </is>
       </c>
-      <c r="C127" t="n">
+      <c r="C127" t="inlineStr"/>
+      <c r="D127" t="n">
         <v>230</v>
       </c>
-      <c r="D127" t="inlineStr">
+      <c r="E127" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3111,15 +3343,16 @@
           <t>Suðurvellir 1</t>
         </is>
       </c>
-      <c r="C128" t="n">
+      <c r="C128" t="inlineStr"/>
+      <c r="D128" t="n">
         <v>230</v>
       </c>
-      <c r="D128" t="inlineStr">
+      <c r="E128" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3132,15 +3365,16 @@
           <t>Suðurvellir 7</t>
         </is>
       </c>
-      <c r="C129" t="n">
+      <c r="C129" t="inlineStr"/>
+      <c r="D129" t="n">
         <v>230</v>
       </c>
-      <c r="D129" t="inlineStr">
+      <c r="E129" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3153,15 +3387,20 @@
           <t>Sóltún 7, íbúð 0101</t>
         </is>
       </c>
-      <c r="C130" t="n">
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
         <v>230</v>
       </c>
-      <c r="D130" t="inlineStr">
+      <c r="E130" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3174,15 +3413,20 @@
           <t>Túngata 12, íbúð 0101</t>
         </is>
       </c>
-      <c r="C131" t="n">
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
         <v>230</v>
       </c>
-      <c r="D131" t="inlineStr">
+      <c r="E131" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3195,15 +3439,16 @@
           <t>Hlíðargata 32</t>
         </is>
       </c>
-      <c r="C132" t="n">
+      <c r="C132" t="inlineStr"/>
+      <c r="D132" t="n">
         <v>245</v>
       </c>
-      <c r="D132" t="inlineStr">
+      <c r="E132" t="inlineStr">
         <is>
           <t>Suðurnesjabær</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -3216,15 +3461,16 @@
           <t>Túngata 16</t>
         </is>
       </c>
-      <c r="C133" t="n">
+      <c r="C133" t="inlineStr"/>
+      <c r="D133" t="n">
         <v>245</v>
       </c>
-      <c r="D133" t="inlineStr">
+      <c r="E133" t="inlineStr">
         <is>
           <t>Suðurnesjabær</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -3237,15 +3483,16 @@
           <t>Bjarkartún 5</t>
         </is>
       </c>
-      <c r="C134" t="n">
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="n">
         <v>250</v>
       </c>
-      <c r="D134" t="inlineStr">
+      <c r="E134" t="inlineStr">
         <is>
           <t>Suðurnesjabær</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3258,15 +3505,16 @@
           <t>Háteigur 5</t>
         </is>
       </c>
-      <c r="C135" t="n">
+      <c r="C135" t="inlineStr"/>
+      <c r="D135" t="n">
         <v>250</v>
       </c>
-      <c r="D135" t="inlineStr">
+      <c r="E135" t="inlineStr">
         <is>
           <t>Suðurnesjabær</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3279,15 +3527,16 @@
           <t>Skagabraut 13</t>
         </is>
       </c>
-      <c r="C136" t="n">
+      <c r="C136" t="inlineStr"/>
+      <c r="D136" t="n">
         <v>250</v>
       </c>
-      <c r="D136" t="inlineStr">
+      <c r="E136" t="inlineStr">
         <is>
           <t>Suðurnesjabær</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3300,15 +3549,16 @@
           <t>Þórshamrar</t>
         </is>
       </c>
-      <c r="C137" t="n">
+      <c r="C137" t="inlineStr"/>
+      <c r="D137" t="n">
         <v>250</v>
       </c>
-      <c r="D137" t="inlineStr">
+      <c r="E137" t="inlineStr">
         <is>
           <t>Suðurnesjabær</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3321,15 +3571,16 @@
           <t>Huldudalur 5</t>
         </is>
       </c>
-      <c r="C138" t="n">
+      <c r="C138" t="inlineStr"/>
+      <c r="D138" t="n">
         <v>260</v>
       </c>
-      <c r="D138" t="inlineStr">
+      <c r="E138" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3342,15 +3593,16 @@
           <t>Kirkjubraut 3</t>
         </is>
       </c>
-      <c r="C139" t="n">
+      <c r="C139" t="inlineStr"/>
+      <c r="D139" t="n">
         <v>260</v>
       </c>
-      <c r="D139" t="inlineStr">
+      <c r="E139" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3363,15 +3615,16 @@
           <t>Laufdalur 51</t>
         </is>
       </c>
-      <c r="C140" t="n">
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="n">
         <v>260</v>
       </c>
-      <c r="D140" t="inlineStr">
+      <c r="E140" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3384,15 +3637,16 @@
           <t>Stapavellir 5</t>
         </is>
       </c>
-      <c r="C141" t="n">
+      <c r="C141" t="inlineStr"/>
+      <c r="D141" t="n">
         <v>260</v>
       </c>
-      <c r="D141" t="inlineStr">
+      <c r="E141" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3405,15 +3659,20 @@
           <t>Bogabraut 963A, íbúð 0204</t>
         </is>
       </c>
-      <c r="C142" t="n">
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>0204</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
         <v>262</v>
       </c>
-      <c r="D142" t="inlineStr">
+      <c r="E142" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3426,15 +3685,20 @@
           <t>Skógarbraut 916C, íbúð 0106</t>
         </is>
       </c>
-      <c r="C143" t="n">
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>0106</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
         <v>262</v>
       </c>
-      <c r="D143" t="inlineStr">
+      <c r="E143" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3447,15 +3711,20 @@
           <t>Skógarbraut 916C, íbúð 0207</t>
         </is>
       </c>
-      <c r="C144" t="n">
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>0207</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
         <v>262</v>
       </c>
-      <c r="D144" t="inlineStr">
+      <c r="E144" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3468,15 +3737,16 @@
           <t>Arnartangi 23</t>
         </is>
       </c>
-      <c r="C145" t="n">
+      <c r="C145" t="inlineStr"/>
+      <c r="D145" t="n">
         <v>270</v>
       </c>
-      <c r="D145" t="inlineStr">
+      <c r="E145" t="inlineStr">
         <is>
           <t>Mosfellsbær</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3489,15 +3759,16 @@
           <t>Krókabyggð 36</t>
         </is>
       </c>
-      <c r="C146" t="n">
+      <c r="C146" t="inlineStr"/>
+      <c r="D146" t="n">
         <v>270</v>
       </c>
-      <c r="D146" t="inlineStr">
+      <c r="E146" t="inlineStr">
         <is>
           <t>Mosfellsbær</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3510,15 +3781,16 @@
           <t>Leirutangi 11A</t>
         </is>
       </c>
-      <c r="C147" t="n">
+      <c r="C147" t="inlineStr"/>
+      <c r="D147" t="n">
         <v>270</v>
       </c>
-      <c r="D147" t="inlineStr">
+      <c r="E147" t="inlineStr">
         <is>
           <t>Mosfellsbær</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3531,15 +3803,16 @@
           <t>Leirutangi 22</t>
         </is>
       </c>
-      <c r="C148" t="n">
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="n">
         <v>270</v>
       </c>
-      <c r="D148" t="inlineStr">
+      <c r="E148" t="inlineStr">
         <is>
           <t>Mosfellsbær</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3552,15 +3825,16 @@
           <t>Leirvogstunga 12</t>
         </is>
       </c>
-      <c r="C149" t="n">
+      <c r="C149" t="inlineStr"/>
+      <c r="D149" t="n">
         <v>270</v>
       </c>
-      <c r="D149" t="inlineStr">
+      <c r="E149" t="inlineStr">
         <is>
           <t>Mosfellsbær</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3573,15 +3847,16 @@
           <t>Litlagerði</t>
         </is>
       </c>
-      <c r="C150" t="n">
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="n">
         <v>270</v>
       </c>
-      <c r="D150" t="inlineStr">
+      <c r="E150" t="inlineStr">
         <is>
           <t>Mosfellsbær</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3594,15 +3869,16 @@
           <t>Reykjavegur 86</t>
         </is>
       </c>
-      <c r="C151" t="n">
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="n">
         <v>270</v>
       </c>
-      <c r="D151" t="inlineStr">
+      <c r="E151" t="inlineStr">
         <is>
           <t>Mosfellsbær</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3615,15 +3891,16 @@
           <t>Ármúli 3</t>
         </is>
       </c>
-      <c r="C152" t="n">
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="n">
         <v>108</v>
       </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E152" t="inlineStr"/>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3636,15 +3913,16 @@
           <t>Flúðasel 67</t>
         </is>
       </c>
-      <c r="C153" t="n">
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="n">
         <v>109</v>
       </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr"/>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3657,15 +3935,16 @@
           <t>Katrínartún 4</t>
         </is>
       </c>
-      <c r="C154" t="n">
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="n">
         <v>105</v>
       </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E154" t="inlineStr"/>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3678,15 +3957,16 @@
           <t>Dalbrekka 56</t>
         </is>
       </c>
-      <c r="C155" t="n">
+      <c r="C155" t="inlineStr"/>
+      <c r="D155" t="n">
         <v>200</v>
       </c>
-      <c r="D155" t="inlineStr">
+      <c r="E155" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3699,15 +3979,16 @@
           <t>Katrínartún 4</t>
         </is>
       </c>
-      <c r="C156" t="n">
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="n">
         <v>105</v>
       </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E156" t="inlineStr"/>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3720,15 +4001,16 @@
           <t>Seinakur 8</t>
         </is>
       </c>
-      <c r="C157" t="n">
+      <c r="C157" t="inlineStr"/>
+      <c r="D157" t="n">
         <v>210</v>
       </c>
-      <c r="D157" t="inlineStr">
+      <c r="E157" t="inlineStr">
         <is>
           <t>Garðabær</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -3741,15 +4023,16 @@
           <t>Ármúli 21</t>
         </is>
       </c>
-      <c r="C158" t="n">
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="n">
         <v>108</v>
       </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>Reykjavík</t>
-        </is>
-      </c>
-      <c r="E158" t="inlineStr"/>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3762,15 +4045,16 @@
           <t>Hafnargata 35</t>
         </is>
       </c>
-      <c r="C159" t="n">
+      <c r="C159" t="inlineStr"/>
+      <c r="D159" t="n">
         <v>230</v>
       </c>
-      <c r="D159" t="inlineStr">
+      <c r="E159" t="inlineStr">
         <is>
           <t>Reykjanesbær</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3783,15 +4067,16 @@
           <t>Kópavogsbraut 88</t>
         </is>
       </c>
-      <c r="C160" t="n">
+      <c r="C160" t="inlineStr"/>
+      <c r="D160" t="n">
         <v>200</v>
       </c>
-      <c r="D160" t="inlineStr">
+      <c r="E160" t="inlineStr">
         <is>
           <t>Kópavogur</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>